<commit_message>
fix: resolve Excel XML load repair error by explicitly setting pageSetup DPI (300) and preventing empty-string sub-cell node creation in merged ranges
</commit_message>
<xml_diff>
--- a/services/attendance/src/scripts/official_a4_test_output.xlsx
+++ b/services/attendance/src/scripts/official_a4_test_output.xlsx
@@ -11,36 +11,39 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="58">
+  <si>
+    <t>Form No. TUHMB-028</t>
+  </si>
+  <si>
+    <t>Technological University ( Hmawbi )</t>
+  </si>
+  <si>
+    <t>Attendance Record ( 2025 - 2026 )</t>
+  </si>
+  <si>
+    <t>V MC</t>
+  </si>
+  <si>
+    <t>ဘာသာရပ် - Industrial Automation II ( McE-52039 )</t>
+  </si>
+  <si>
+    <t>၂၀၂၅ - ၂၀၂၆ ခုနှစ်၊ ဇန်နဝါရီ (Jan) လ</t>
+  </si>
+  <si>
+    <t>ယခုလတက်ချိန် - 36 နာရီ</t>
+  </si>
+  <si>
+    <t>စဉ်</t>
+  </si>
+  <si>
+    <t>ခုံအမှတ်</t>
+  </si>
+  <si>
+    <t>အမည်</t>
+  </si>
   <si>
     <t/>
-  </si>
-  <si>
-    <t>Technological University ( Hmawbi )</t>
-  </si>
-  <si>
-    <t>Attendance Record ( 2025 - 2026 )</t>
-  </si>
-  <si>
-    <t>V MC</t>
-  </si>
-  <si>
-    <t>ဘာသာရပ် - Industrial Automation II ( McE-52039 )</t>
-  </si>
-  <si>
-    <t>၂၀၂၅ - ၂၀၂၆ ခုနှစ်၊ ဇန်နဝါရီ (Jan) လ</t>
-  </si>
-  <si>
-    <t>ယခုလတက်ချိန် - 36 နာရီ</t>
-  </si>
-  <si>
-    <t>စဉ်</t>
-  </si>
-  <si>
-    <t>ခုံအမှတ်</t>
-  </si>
-  <si>
-    <t>အမည်</t>
   </si>
   <si>
     <t>တက်ချိန်ပေါင်း</t>
@@ -188,7 +191,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -197,26 +200,29 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="9"/>
+      <sz val="8"/>
     </font>
     <font>
       <b/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="12"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
     </font>
     <font>
-      <sz val="10"/>
+      <b/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <sz val="9"/>
     </font>
     <font>
       <b/>
-      <sz val="9"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <sz val="8.5"/>
     </font>
     <font>
       <i/>
@@ -258,7 +264,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -280,13 +286,16 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -631,77 +640,16 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y35"/>
+  <dimension ref="A1:Y34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="22" width="2.2" customWidth="1"/>
-    <col min="23" max="25" width="3.5" customWidth="1"/>
+    <col min="1" max="1" width="3.5" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="22" width="1.6" customWidth="1"/>
+    <col min="23" max="25" width="3.2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" t="s">
-        <v>0</v>
-      </c>
-      <c r="I1" t="s">
-        <v>0</v>
-      </c>
-      <c r="J1" t="s">
-        <v>0</v>
-      </c>
-      <c r="K1" t="s">
-        <v>0</v>
-      </c>
-      <c r="L1" t="s">
-        <v>0</v>
-      </c>
-      <c r="M1" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" t="s">
-        <v>0</v>
-      </c>
-      <c r="O1" t="s">
-        <v>0</v>
-      </c>
-      <c r="P1" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>0</v>
-      </c>
-      <c r="R1" t="s">
-        <v>0</v>
-      </c>
-      <c r="S1" t="s">
-        <v>0</v>
-      </c>
-      <c r="T1" t="s">
-        <v>0</v>
-      </c>
+    <row r="1" spans="21:25" x14ac:dyDescent="0.25">
       <c r="U1" s="1" t="s">
         <v>0</v>
       </c>
@@ -773,36 +721,6 @@
         <v>3</v>
       </c>
       <c r="B4" s="4"/>
-      <c r="C4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" t="s">
-        <v>0</v>
-      </c>
-      <c r="F4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G4" t="s">
-        <v>0</v>
-      </c>
-      <c r="H4" t="s">
-        <v>0</v>
-      </c>
-      <c r="I4" t="s">
-        <v>0</v>
-      </c>
-      <c r="J4" t="s">
-        <v>0</v>
-      </c>
-      <c r="K4" t="s">
-        <v>0</v>
-      </c>
-      <c r="L4" t="s">
-        <v>0</v>
-      </c>
       <c r="M4" s="5" t="s">
         <v>4</v>
       </c>
@@ -850,2072 +768,2036 @@
       <c r="X5" s="5"/>
       <c r="Y5" s="5"/>
     </row>
-    <row r="7" ht="70" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+    <row r="6" ht="60" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="K7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="L7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="M7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="N7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="O7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="P7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="R7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="S7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="T7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="U7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="V7" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="W7" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="X7" s="8" t="s">
+      <c r="D6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="R6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="S6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="T6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="U6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="V6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="W6" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="Y7" s="8" t="s">
+      <c r="X6" s="8" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y6" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="L7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="N7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="O7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="P7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="R7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="S7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="T7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="U7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="V7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="W7" s="9">
+        <f>=COUNTIF(D7:V7, "✓") * 3</f>
+      </c>
+      <c r="X7" s="9">
+        <f>=(COUNTA(D$6:V$6) - COUNTIF(D7:V7, "✓")) * 3</f>
+      </c>
+      <c r="Y7" s="9">
+        <f>=IF((W7+X7)&gt;0, ROUND((W7/(W7+X7))*100, 1) &amp; "%", "100%")</f>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V8" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W8" s="9">
         <f>=COUNTIF(D8:V8, "✓") * 3</f>
       </c>
       <c r="X8" s="9">
-        <f>=(COUNTA(D$7:V$7) - COUNTIF(D8:V8, "✓")) * 3</f>
+        <f>=(COUNTA(D$6:V$6) - COUNTIF(D8:V8, "✓")) * 3</f>
       </c>
       <c r="Y8" s="9">
         <f>=IF((W8+X8)&gt;0, ROUND((W8/(W8+X8))*100, 1) &amp; "%", "100%")</f>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="9" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V9" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W9" s="9">
         <f>=COUNTIF(D9:V9, "✓") * 3</f>
       </c>
       <c r="X9" s="9">
-        <f>=(COUNTA(D$7:V$7) - COUNTIF(D9:V9, "✓")) * 3</f>
+        <f>=(COUNTA(D$6:V$6) - COUNTIF(D9:V9, "✓")) * 3</f>
       </c>
       <c r="Y9" s="9">
         <f>=IF((W9+X9)&gt;0, ROUND((W9/(W9+X9))*100, 1) &amp; "%", "100%")</f>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="10" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V10" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W10" s="9">
         <f>=COUNTIF(D10:V10, "✓") * 3</f>
       </c>
       <c r="X10" s="9">
-        <f>=(COUNTA(D$7:V$7) - COUNTIF(D10:V10, "✓")) * 3</f>
+        <f>=(COUNTA(D$6:V$6) - COUNTIF(D10:V10, "✓")) * 3</f>
       </c>
       <c r="Y10" s="9">
         <f>=IF((W10+X10)&gt;0, ROUND((W10/(W10+X10))*100, 1) &amp; "%", "100%")</f>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="11" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V11" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W11" s="9">
         <f>=COUNTIF(D11:V11, "✓") * 3</f>
       </c>
       <c r="X11" s="9">
-        <f>=(COUNTA(D$7:V$7) - COUNTIF(D11:V11, "✓")) * 3</f>
+        <f>=(COUNTA(D$6:V$6) - COUNTIF(D11:V11, "✓")) * 3</f>
       </c>
       <c r="Y11" s="9">
         <f>=IF((W11+X11)&gt;0, ROUND((W11/(W11+X11))*100, 1) &amp; "%", "100%")</f>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="12" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V12" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W12" s="9">
         <f>=COUNTIF(D12:V12, "✓") * 3</f>
       </c>
       <c r="X12" s="9">
-        <f>=(COUNTA(D$7:V$7) - COUNTIF(D12:V12, "✓")) * 3</f>
+        <f>=(COUNTA(D$6:V$6) - COUNTIF(D12:V12, "✓")) * 3</f>
       </c>
       <c r="Y12" s="9">
         <f>=IF((W12+X12)&gt;0, ROUND((W12/(W12+X12))*100, 1) &amp; "%", "100%")</f>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="13" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V13" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W13" s="9">
         <f>=COUNTIF(D13:V13, "✓") * 3</f>
       </c>
       <c r="X13" s="9">
-        <f>=(COUNTA(D$7:V$7) - COUNTIF(D13:V13, "✓")) * 3</f>
+        <f>=(COUNTA(D$6:V$6) - COUNTIF(D13:V13, "✓")) * 3</f>
       </c>
       <c r="Y13" s="9">
         <f>=IF((W13+X13)&gt;0, ROUND((W13/(W13+X13))*100, 1) &amp; "%", "100%")</f>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="14" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V14" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W14" s="9">
         <f>=COUNTIF(D14:V14, "✓") * 3</f>
       </c>
       <c r="X14" s="9">
-        <f>=(COUNTA(D$7:V$7) - COUNTIF(D14:V14, "✓")) * 3</f>
+        <f>=(COUNTA(D$6:V$6) - COUNTIF(D14:V14, "✓")) * 3</f>
       </c>
       <c r="Y14" s="9">
         <f>=IF((W14+X14)&gt;0, ROUND((W14/(W14+X14))*100, 1) &amp; "%", "100%")</f>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="15" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V15" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W15" s="9">
         <f>=COUNTIF(D15:V15, "✓") * 3</f>
       </c>
       <c r="X15" s="9">
-        <f>=(COUNTA(D$7:V$7) - COUNTIF(D15:V15, "✓")) * 3</f>
+        <f>=(COUNTA(D$6:V$6) - COUNTIF(D15:V15, "✓")) * 3</f>
       </c>
       <c r="Y15" s="9">
         <f>=IF((W15+X15)&gt;0, ROUND((W15/(W15+X15))*100, 1) &amp; "%", "100%")</f>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="16" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V16" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W16" s="9">
         <f>=COUNTIF(D16:V16, "✓") * 3</f>
       </c>
       <c r="X16" s="9">
-        <f>=(COUNTA(D$7:V$7) - COUNTIF(D16:V16, "✓")) * 3</f>
+        <f>=(COUNTA(D$6:V$6) - COUNTIF(D16:V16, "✓")) * 3</f>
       </c>
       <c r="Y16" s="9">
         <f>=IF((W16+X16)&gt;0, ROUND((W16/(W16+X16))*100, 1) &amp; "%", "100%")</f>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="17" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V17" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W17" s="9">
         <f>=COUNTIF(D17:V17, "✓") * 3</f>
       </c>
       <c r="X17" s="9">
-        <f>=(COUNTA(D$7:V$7) - COUNTIF(D17:V17, "✓")) * 3</f>
+        <f>=(COUNTA(D$6:V$6) - COUNTIF(D17:V17, "✓")) * 3</f>
       </c>
       <c r="Y17" s="9">
         <f>=IF((W17+X17)&gt;0, ROUND((W17/(W17+X17))*100, 1) &amp; "%", "100%")</f>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="18" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V18" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W18" s="9">
         <f>=COUNTIF(D18:V18, "✓") * 3</f>
       </c>
       <c r="X18" s="9">
-        <f>=(COUNTA(D$7:V$7) - COUNTIF(D18:V18, "✓")) * 3</f>
+        <f>=(COUNTA(D$6:V$6) - COUNTIF(D18:V18, "✓")) * 3</f>
       </c>
       <c r="Y18" s="9">
         <f>=IF((W18+X18)&gt;0, ROUND((W18/(W18+X18))*100, 1) &amp; "%", "100%")</f>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="19" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V19" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W19" s="9">
         <f>=COUNTIF(D19:V19, "✓") * 3</f>
       </c>
       <c r="X19" s="9">
-        <f>=(COUNTA(D$7:V$7) - COUNTIF(D19:V19, "✓")) * 3</f>
+        <f>=(COUNTA(D$6:V$6) - COUNTIF(D19:V19, "✓")) * 3</f>
       </c>
       <c r="Y19" s="9">
         <f>=IF((W19+X19)&gt;0, ROUND((W19/(W19+X19))*100, 1) &amp; "%", "100%")</f>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="20" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V20" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W20" s="9">
         <f>=COUNTIF(D20:V20, "✓") * 3</f>
       </c>
       <c r="X20" s="9">
-        <f>=(COUNTA(D$7:V$7) - COUNTIF(D20:V20, "✓")) * 3</f>
+        <f>=(COUNTA(D$6:V$6) - COUNTIF(D20:V20, "✓")) * 3</f>
       </c>
       <c r="Y20" s="9">
         <f>=IF((W20+X20)&gt;0, ROUND((W20/(W20+X20))*100, 1) &amp; "%", "100%")</f>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="21" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>54</v>
+        <v>10</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U21" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V21" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="W21" s="9">
-        <f>=COUNTIF(D21:V21, "✓") * 3</f>
-      </c>
-      <c r="X21" s="9">
-        <f>=(COUNTA(D$7:V$7) - COUNTIF(D21:V21, "✓")) * 3</f>
-      </c>
-      <c r="Y21" s="9">
-        <f>=IF((W21+X21)&gt;0, ROUND((W21/(W21+X21))*100, 1) &amp; "%", "100%")</f>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="W21" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="X21" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y21" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="X22" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Y22" s="9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="X23" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Y23" s="9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="X24" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Y24" s="9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="X25" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Y25" s="9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="X26" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Y26" s="9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="X27" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Y27" s="9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="X28" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Y28" s="9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="X29" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Y29" s="9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="X30" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Y30" s="9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="T31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="U31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="V31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="X31" s="9" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Y31" s="9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="C32" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="E32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="G32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="H32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="I32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="J32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="K32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="L32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="M32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="N32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="O32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="P32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="R32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="S32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="T32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="U32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="V32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="W32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="X32" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="Y32" s="9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>0</v>
-      </c>
-      <c r="B34" t="s">
-        <v>0</v>
-      </c>
-      <c r="C34" t="s">
-        <v>0</v>
-      </c>
-      <c r="D34" t="s">
-        <v>0</v>
-      </c>
-      <c r="E34" t="s">
-        <v>0</v>
-      </c>
-      <c r="F34" t="s">
-        <v>0</v>
-      </c>
-      <c r="G34" t="s">
-        <v>0</v>
-      </c>
-      <c r="H34" t="s">
-        <v>0</v>
-      </c>
-      <c r="I34" t="s">
-        <v>0</v>
-      </c>
-      <c r="J34" t="s">
-        <v>0</v>
-      </c>
-      <c r="K34" t="s">
-        <v>0</v>
-      </c>
-      <c r="L34" t="s">
-        <v>0</v>
-      </c>
-      <c r="M34" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="N34" s="1"/>
-      <c r="O34" s="1"/>
-      <c r="P34" s="1"/>
-      <c r="Q34" s="1"/>
-      <c r="R34" s="1"/>
-      <c r="S34" s="1"/>
-      <c r="T34" s="1"/>
-      <c r="U34" s="1"/>
-      <c r="V34" s="1"/>
-      <c r="W34" s="1"/>
-      <c r="X34" s="1"/>
-      <c r="Y34" s="1"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="13:25" x14ac:dyDescent="0.25">
+      <c r="M33" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="11"/>
-      <c r="G35" s="11"/>
-      <c r="H35" s="11"/>
+      <c r="N33" s="11"/>
+      <c r="O33" s="11"/>
+      <c r="P33" s="11"/>
+      <c r="Q33" s="11"/>
+      <c r="R33" s="11"/>
+      <c r="S33" s="11"/>
+      <c r="T33" s="11"/>
+      <c r="U33" s="11"/>
+      <c r="V33" s="11"/>
+      <c r="W33" s="11"/>
+      <c r="X33" s="11"/>
+      <c r="Y33" s="11"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B34" s="12"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -2926,8 +2808,8 @@
     <mergeCell ref="M4:Y4"/>
     <mergeCell ref="A5:L5"/>
     <mergeCell ref="M5:Y5"/>
-    <mergeCell ref="M34:Y34"/>
-    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="M33:Y33"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>